<commit_message>
chore(content): update dates to 2026-09-07, refresh challenger models
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -340,6 +340,7 @@
     <col min="15" max="15" width="19" customWidth="1"/>
     <col min="16" max="16" width="19" customWidth="1"/>
     <col min="17" max="17" width="19" customWidth="1"/>
+    <col min="18" max="18" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">
@@ -428,6 +429,11 @@
           <t>首页展示顺序</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>父记录</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="25.5" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -513,6 +519,7 @@
           <t>2</t>
         </is>
       </c>
+      <c r="R2"/>
     </row>
     <row r="3" ht="25.5" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -598,6 +605,7 @@
           <t>1</t>
         </is>
       </c>
+      <c r="R3"/>
     </row>
     <row r="4" ht="25.5" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -677,6 +685,7 @@
           <t>3</t>
         </is>
       </c>
+      <c r="R4"/>
     </row>
     <row r="5" ht="25.5" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -752,6 +761,7 @@
       <c r="O5"/>
       <c r="P5"/>
       <c r="Q5"/>
+      <c r="R5"/>
     </row>
     <row r="6" ht="25.5" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -817,13 +827,14 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>私部署版：BISHENG + GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/LongCat 2.0/Minimax M3/DeepSeek V4 Pro/Step 3.7 Flash/Ling 3.0 flash</t>
+          <t>私部署版：BISHENG + GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/LongCat 2.0/Minimax M3/DeepSeek V4 Pro/Step 3.7 Flash/Ling 3.0 flash/Spark X2.5</t>
         </is>
       </c>
       <c r="N6"/>
       <c r="O6"/>
       <c r="P6"/>
       <c r="Q6"/>
+      <c r="R6"/>
     </row>
     <row r="7" ht="25.5" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -897,6 +908,7 @@
       <c r="O7"/>
       <c r="P7"/>
       <c r="Q7"/>
+      <c r="R7"/>
     </row>
     <row r="8" ht="25.5" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -969,6 +981,7 @@
       <c r="O8"/>
       <c r="P8"/>
       <c r="Q8"/>
+      <c r="R8"/>
     </row>
     <row r="9" ht="25.5" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -1040,6 +1053,7 @@
       <c r="O9"/>
       <c r="P9"/>
       <c r="Q9"/>
+      <c r="R9"/>
     </row>
     <row r="10" ht="25.5" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -1113,6 +1127,7 @@
       <c r="O10"/>
       <c r="P10"/>
       <c r="Q10"/>
+      <c r="R10"/>
     </row>
     <row r="11" ht="25.5" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -1185,6 +1200,7 @@
       <c r="O11"/>
       <c r="P11"/>
       <c r="Q11"/>
+      <c r="R11"/>
     </row>
     <row r="12" ht="25.5" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -1257,6 +1273,7 @@
       <c r="O12"/>
       <c r="P12"/>
       <c r="Q12"/>
+      <c r="R12"/>
     </row>
     <row r="13" ht="25.5" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -1329,6 +1346,7 @@
       <c r="O13"/>
       <c r="P13"/>
       <c r="Q13"/>
+      <c r="R13"/>
     </row>
     <row r="14" ht="25.5" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -1401,6 +1419,7 @@
       <c r="O14"/>
       <c r="P14"/>
       <c r="Q14"/>
+      <c r="R14"/>
     </row>
     <row r="15" ht="25.5" customHeight="1">
       <c r="A15"/>
@@ -1420,6 +1439,7 @@
       <c r="O15"/>
       <c r="P15"/>
       <c r="Q15"/>
+      <c r="R15"/>
     </row>
     <row r="16" ht="25.5" customHeight="1">
       <c r="A16"/>
@@ -1439,6 +1459,7 @@
       <c r="O16"/>
       <c r="P16"/>
       <c r="Q16"/>
+      <c r="R16"/>
     </row>
   </sheetData>
   <dataValidations count="5">

</xml_diff>

<commit_message>
chore(content): update dates to 2026-09-14
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -1461,21 +1461,41 @@
       <c r="Q16"/>
       <c r="R16"/>
     </row>
+    <row r="17" ht="25.5" customHeight="1">
+      <c r="A17"/>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="H17"/>
+      <c r="I17"/>
+      <c r="J17"/>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17"/>
+      <c r="O17"/>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation allowBlank="false" sqref="E2:E15" type="list">
+    <dataValidation allowBlank="false" sqref="E2:E16" type="list">
       <formula1>"已验证,验证中"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="I2:I15" type="list">
+    <dataValidation allowBlank="false" sqref="I2:I16" type="list">
       <formula1>"一周,1~2天"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="J2:J15" type="list">
+    <dataValidation allowBlank="false" sqref="J2:J16" type="list">
       <formula1>"较高,很高,中等,较低"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="K2:K15" type="list">
+    <dataValidation allowBlank="false" sqref="K2:K16" type="list">
       <formula1>"较高,较低"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="L2:L15" type="list">
+    <dataValidation allowBlank="false" sqref="L2:L16" type="list">
       <formula1>"较优,中等"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(content): update dates to 2026-09-22, refresh challenger models
- Update "Last Updated" dates from 2026-09-14 to 2026-09-22 across all arena overviews
- Upgrade MiMo V2.5 Pro to MiMo V2.6 Pro in challenger lineups (arenas 1, 4, 7)
- Add Confucius4-R2T2 to the ASR model list for arena 4
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Hermes Agent + GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/MiMo V2.5 Pro+ Metaso</t>
+          <t>私部署版：Hermes Agent + MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>私部署版：OpenClaw + GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/DeepSeek V4 Pro/MiMo V2.5 Pro + FFmpeg + MOSS-Audio/FireRedASR/Qwen3-ASR/GLM-ASR/MiMo-V2.5-ASR + MOSS-TTS/VoxCPM/Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS/Step-Audio-TTS/Confucius4-TTS/IndexTTS-2.5/Dots-TTS/FireRedTTS3</t>
+          <t>私部署版：OpenClaw + MiMo V2.6 Pro/GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/DeepSeek V4 Pro + FFmpeg + MOSS-Audio/FireRedASR/Qwen3-ASR/GLM-ASR/MiMo-V2.5-ASR/Confucius4-R2T2 + MOSS-TTS/VoxCPM/Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS/Step-Audio-TTS/Confucius4-TTS/IndexTTS-2.5/Dots-TTS/FireRedTTS3</t>
         </is>
       </c>
       <c r="N5"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/Kimi K2.7 Code/DeepSeek V4 Pro/MiMo V2.5 Pro</t>
+          <t>私部署版：Claude Code + MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/Kimi K2.7 Code/DeepSeek V4 Pro</t>
         </is>
       </c>
       <c r="N8"/>

</xml_diff>

<commit_message>
chore(content): update dates to 2026-09-28
- Update "Last Updated" dates from 2026-09-22 to 2026-09-28 across all arena overviews
- Update List of Arenas.xlsx index
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -1481,21 +1481,41 @@
       <c r="Q17"/>
       <c r="R17"/>
     </row>
+    <row r="18" ht="25.5" customHeight="1">
+      <c r="A18"/>
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18"/>
+      <c r="I18"/>
+      <c r="J18"/>
+      <c r="K18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18"/>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation allowBlank="false" sqref="E2:E16" type="list">
+    <dataValidation allowBlank="false" sqref="E2:E17" type="list">
       <formula1>"已验证,验证中"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="I2:I16" type="list">
+    <dataValidation allowBlank="false" sqref="I2:I17" type="list">
       <formula1>"一周,1~2天"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="J2:J16" type="list">
+    <dataValidation allowBlank="false" sqref="J2:J17" type="list">
       <formula1>"较高,很高,中等,较低"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="K2:K16" type="list">
+    <dataValidation allowBlank="false" sqref="K2:K17" type="list">
       <formula1>"较高,较低"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="L2:L16" type="list">
+    <dataValidation allowBlank="false" sqref="L2:L17" type="list">
       <formula1>"较优,中等"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(content): update dates to 2026-10-19, refresh challenger models
- Update "Last Updated" dates from 2026-10-12 to 2026-10-19 across all arena overviews
- Replace DeepSeek V4 Pro with DeepSeek V4.1 Flash in challenger lineups (arenas 2, 4, 5, 7)
- Update Ling 3.0 flash to Ling 3.1 flash in arena 5 challenger list
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>云端版：Lovable + GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/MiniMax M3/DeepSeek V4 Pro+ Claude Code</t>
+          <t>云端版：Lovable + GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/MiniMax M3/DeepSeek V4.1 Flash+ Claude Code</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>私部署版：OpenClaw + MiMo V2.6 Pro/GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/DeepSeek V4 Pro + FFmpeg + MOSS-Audio/FireRedASR/Qwen3-ASR/GLM-ASR/MiMo-V2.5-ASR/Confucius4-R2T2 + MOSS-TTS/VoxCPM/Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS/Step-Audio-TTS/Confucius4-TTS/IndexTTS-2.5/Dots-TTS/FireRedTTS3</t>
+          <t>私部署版：OpenClaw + MiMo V2.6 Pro/GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/DeepSeek V4.1 Flash + FFmpeg + MOSS-Audio/FireRedASR/Qwen3-ASR/GLM-ASR/MiMo-V2.5-ASR/Confucius4-R2T2 + MOSS-TTS/VoxCPM/Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS/Step-Audio-TTS/Confucius4-TTS/IndexTTS-2.5/Dots-TTS/FireRedTTS3</t>
         </is>
       </c>
       <c r="N5"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>私部署版：BISHENG + GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/LongCat 2.0/Minimax M3/DeepSeek V4 Pro/Step 5 preview/Ling 3.0 flash/Spark X2.5</t>
+          <t>私部署版：BISHENG + GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/LongCat 2.0/Minimax M3/DeepSeek V4.1 Flash/Step 5 preview/Ling 3.1 flash/Spark X2.5</t>
         </is>
       </c>
       <c r="N6"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/Kimi K2.7 Code/DeepSeek V4 Pro</t>
+          <t>私部署版：Claude Code + MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/Kimi K2.7 Code/DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="N8"/>

</xml_diff>

<commit_message>
chore(content): update dates to 2026-10-26, refresh challenger models
- Update "Last Updated" dates from 2026-10-19 to 2026-10-26 across all arena overviews
- Add Kimi K3.1 Pro, MiniMax M3.1 Flash/Pro, and DeepSeek V4.1 Flash to challenger lineups; drop Kimi K3, Minimax M3, DeepSeek V4 Pro, GLM 5.2, and Qwen 3.7
- Add Ming-3.0-ASR-Tiny and Ming-3.0-TTS to arena 4 speech stack; upgrade Spark X2.5 to Spark X2.6 in arena 5
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Hermes Agent + MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview+ Metaso</t>
+          <t>私部署版：Hermes Agent + Kimi K3.1 Pro/MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Hy4 preview+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>云端版：Lovable + GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/MiniMax M3/DeepSeek V4.1 Flash+ Claude Code</t>
+          <t>云端版：Lovable + Kimi K3.1 Pro/MiniMax M3.1 Flash/DeepSeek V4.1 Flash/GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code+ Claude Code</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>私部署版：PI Agent+  GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K3/Minimax M3/DeepSeek V4 Pro + Docling OCR/Unlimited-OCR + YAML Workflow + Skills</t>
+          <t>私部署版：PI Agent+ Kimi K3.1 Pro/MiniMax M3.1 Flash/DeepSeek V4.1 Flash/GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0 + Docling OCR/Unlimited-OCR + YAML Workflow + Skills</t>
         </is>
       </c>
       <c r="N4"/>
@@ -754,7 +754,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>私部署版：OpenClaw + MiMo V2.6 Pro/GLM 5.3/Kimi K3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code/DeepSeek V4.1 Flash + FFmpeg + MOSS-Audio/FireRedASR/Qwen3-ASR/GLM-ASR/MiMo-V2.5-ASR/Confucius4-R2T2 + MOSS-TTS/VoxCPM/Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS/Step-Audio-TTS/Confucius4-TTS/IndexTTS-2.5/Dots-TTS/FireRedTTS3</t>
+          <t>私部署版：OpenClaw + Kimi K3.1 Pro/DeepSeek V4.1 Flash/MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code + FFmpeg + MOSS-Audio/FireRedASR/Qwen3-ASR/GLM-ASR/MiMo-V2.5-ASR/Confucius4-R2T2/Ming-3.0-ASR-Tiny + MOSS-TTS/VoxCPM/Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS/Step-Audio-TTS/Confucius4-TTS/IndexTTS-2.5/Dots-TTS/FireRedTTS3/Ming-3.0-TTS</t>
         </is>
       </c>
       <c r="N5"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>私部署版：BISHENG + GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/LongCat 2.0/Minimax M3/DeepSeek V4.1 Flash/Step 5 preview/Ling 3.1 flash/Spark X2.5</t>
+          <t>私部署版：BISHENG + Kimi K3.1 Pro/MiniMax M3.1 Pro/DeepSeek V4.1 Flash/GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Step 5 preview/Ling 3.1 flash/Spark X2.6</t>
         </is>
       </c>
       <c r="N6"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + MiMo V2.6 Pro/GLM 5.3/Qwen3.8 Max/Kimi K3/Hy4 preview/Kimi K2.7 Code/DeepSeek V4.1 Flash</t>
+          <t>私部署版：Claude Code + Kimi K3.1 Pro/MiMo V2.6 Pro/DeepSeek V4.1 Flash/GLM 5.3/Qwen3.8 Max/Hy4 preview/Kimi K2.7 Code</t>
         </is>
       </c>
       <c r="N8"/>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>私部署版：Coze +  GLM 5.3/Hy4 preview/LongCat 2.0/Kimi K3/Kimi K2.7 Code/GLM 5.2/Minimax M3/Qwen 3.7/DeepSeek V4 Pro</t>
+          <t>私部署版：Coze +  Kimi K3.1 Pro/MiniMax M3.1 Flash/DeepSeek V4.1 Flash/GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K2.7 Code</t>
         </is>
       </c>
       <c r="N12"/>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +   GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K3/Minimax M3/DeepSeek V4 Pro  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain + Kimi K3.1 Pro/MiniMax M3.1 Flash/DeepSeek V4.1 Flash/GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N13"/>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +   GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0/Kimi K3/Minimax M3/DeepSeek V4 Pro  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain + Kimi K3.1 Pro/MiniMax M3.1 Flash/DeepSeek V4.1 Flash/GLM 5.3/Qwen3.8 Max/Hy4 preview/LongCat 2.0  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N14"/>

</xml_diff>